<commit_message>
Add governed Vendor import normalization contract
</commit_message>
<xml_diff>
--- a/public/templates/vendors/vendor_import_template_blank.xlsx
+++ b/public/templates/vendors/vendor_import_template_blank.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:Q9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,6 +446,12 @@
       <c r="O1" t="str">
         <v/>
       </c>
+      <c r="P1" t="str">
+        <v/>
+      </c>
+      <c r="Q1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -493,6 +499,12 @@
       <c r="O2" t="str">
         <v/>
       </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -538,6 +550,12 @@
         <v/>
       </c>
       <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v/>
       </c>
     </row>
@@ -587,6 +605,12 @@
       <c r="O4" t="str">
         <v>Display Order</v>
       </c>
+      <c r="P4" t="str">
+        <v>Show on Member Dashboard</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Allow Service Requests</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -634,6 +658,12 @@
       <c r="O5" t="str">
         <v/>
       </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -681,6 +711,12 @@
       <c r="O6" t="str">
         <v/>
       </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -728,6 +764,12 @@
       <c r="O7" t="str">
         <v/>
       </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -775,6 +817,12 @@
       <c r="O8" t="str">
         <v/>
       </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -822,17 +870,23 @@
       <c r="O9" t="str">
         <v/>
       </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1133,17 +1187,51 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>Show on Member Dashboard</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Optional</v>
+      </c>
+      <c r="C22" t="str">
+        <v>boolean_yes_no</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Per-event dashboard-display flag. Maps to the governed event_vendors.show_on_member_dashboard field. Blank preserves the existing Event-Vendor value when Stage 5B execution is implemented.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Allow Service Requests</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Optional</v>
+      </c>
+      <c r="C23" t="str">
+        <v>boolean_yes_no</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Per-event service-request flag. Maps to the governed event_vendors.allow_service_requests field. Blank preserves the existing Event-Vendor value when Stage 5B execution is implemented.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>The sample file can be saved as either XLSX or CSV and used as a model.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>